<commit_message>
Add source attribution script and outputs; update plan and changelog
</commit_message>
<xml_diff>
--- a/my_samples/02 obsidian einan natufian 23.2.17.xlsx
+++ b/my_samples/02 obsidian einan natufian 23.2.17.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\01_ארכיאולוגיה\01_אוניברסיטת חיפה\1_תשפו\אובסידיאן\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\code\obsidian\my_samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ECB3AD3-6A4D-467E-A036-F3D6FFD98118}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE47F5DD-5389-4496-91DF-324CE0CB3386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{0FEE8330-34BC-4883-8F9F-C62D82234DC3}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2227" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2227" uniqueCount="154">
   <si>
     <t>Index</t>
   </si>
@@ -494,6 +494,9 @@
   </si>
   <si>
     <t>Date</t>
+  </si>
+  <si>
+    <t>Dark colored flint</t>
   </si>
 </sst>
 </file>
@@ -13816,7 +13819,7 @@
       <c r="F20" s="14"/>
       <c r="H20" s="14"/>
       <c r="I20" s="14" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="J20" s="14"/>
       <c r="K20" s="11" t="s">

</xml_diff>